<commit_message>
Fill op-eds, policy briefs and project details from research
- Op-eds and blogs: a working link for all 23, corrected outlets, dates and
  author order, and summaries in the same style as the publications.
- Policy briefs: authors, date, three recommendations, issue, evidence and
  a link to the underlying research for all six. Recommendations drafted
  from findings are flagged in each brief's notes for author review.
- Projects: descriptions for 13 of 15, with verified years and partners.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HC9YdbS4ZuWPUdtCTLm1r5
</commit_message>
<xml_diff>
--- a/docs/content-input/RITA-website-content-to-fill.xlsx
+++ b/docs/content-input/RITA-website-content-to-fill.xlsx
@@ -20,8 +20,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1 Institute &amp; legal'!$A$2:$D$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 People'!$A$2:$D$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Publications'!$A$2:$V$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 People'!$A$2:$D$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Publications'!$A$2:$V$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4 Policy Insights'!$A$2:$L$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Op-eds &amp; blogs'!$A$2:$K$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6 Policy briefs'!$A$2:$M$9</definedName>
@@ -2615,7 +2615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3166,7 +3166,7 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Fellows, associates and staff to list (only with their written consent)</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B32" s="14" t="n"/>
@@ -3176,17 +3176,17 @@
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>Solomon Owusu</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Short bio (about 60 words)</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr"/>
@@ -3194,17 +3194,17 @@
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>Woubet Kassa</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Long bio (about 150 words): confirm or correct the current one</t>
         </is>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>Marcel Kempers curates and runs the RITA website. His research looks at e-mobility and informal transport work in African cities, including electric motorcycle taxis (boda bodas) in Nairobi. MSc, Delft University of Technology.</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr"/>
@@ -3212,17 +3212,17 @@
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>Emmanuel B. Mensah</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Role title</t>
         </is>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>Curator &amp; website lead</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr"/>
@@ -3230,17 +3230,17 @@
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>Rexford Asiamah</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Base (city)</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr"/>
@@ -3248,17 +3248,17 @@
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>Christian Urom</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Email to show on profile</t>
         </is>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
@@ -3266,17 +3266,17 @@
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
         <is>
-          <t>Maty Konte</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>LinkedIn URL</t>
         </is>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr"/>
@@ -3284,17 +3284,17 @@
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>Fiona Tregenna</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Google Scholar URL</t>
         </is>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr"/>
@@ -3302,17 +3302,17 @@
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t>Antonio Andreoni</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>ORCID iD</t>
         </is>
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr"/>
@@ -3320,17 +3320,17 @@
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>Shingie Chisoro</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Personal website</t>
         </is>
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr"/>
@@ -3338,17 +3338,17 @@
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>Jason Bell</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Focus tags (5 keywords)</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>E-mobility · Boda bodas · Nairobi · Informal work · Transport</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr"/>
@@ -3356,17 +3356,17 @@
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>Julius Nyamwena</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Topics for media comment</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr"/>
@@ -3374,17 +3374,17 @@
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
         <is>
-          <t>Keyi Tang</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Awards (confirm)</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr"/>
@@ -3392,55 +3392,299 @@
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t>Xiaolan Fu</t>
+          <t>Marcel Kempers</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
+          <t>Portrait photo sent? (4:5, at least 1600×2000 px, with photo release)</t>
         </is>
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>Frequent co-author (not listed on the site)</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="15" t="inlineStr">
-        <is>
-          <t>Erika Kraemer-Mbula</t>
-        </is>
-      </c>
-      <c r="B46" s="15" t="inlineStr">
-        <is>
-          <t>Invite as associate? (Yes / No) + role, email</t>
-        </is>
-      </c>
-      <c r="C46" s="15" t="inlineStr">
-        <is>
-          <t>Frequent co-author (not listed on the site)</t>
-        </is>
-      </c>
-      <c r="D46" s="16" t="inlineStr"/>
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>Fellows, associates and staff to list (only with their written consent)</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="n"/>
+      <c r="C46" s="14" t="n"/>
+      <c r="D46" s="14" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="15" t="inlineStr">
         <is>
+          <t>Solomon Owusu</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>Woubet Kassa</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>Emmanuel B. Mensah</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>Rexford Asiamah</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>Christian Urom</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="15" t="inlineStr">
+        <is>
+          <t>Maty Konte</t>
+        </is>
+      </c>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>Fiona Tregenna</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C53" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="15" t="inlineStr">
+        <is>
+          <t>Antonio Andreoni</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="15" t="inlineStr">
+        <is>
+          <t>Shingie Chisoro</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>Jason Bell</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>Julius Nyamwena</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>Keyi Tang</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C58" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>Xiaolan Fu</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="15" t="inlineStr">
+        <is>
+          <t>Erika Kraemer-Mbula</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>Invite as associate? (Yes / No) + role, email</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>Frequent co-author (not listed on the site)</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
           <t>(Add any other person)</t>
         </is>
       </c>
-      <c r="B47" s="15" t="inlineStr">
+      <c r="B61" s="15" t="inlineStr">
         <is>
           <t>Name, group (fellow / associate / staff), role, base, email</t>
         </is>
       </c>
-      <c r="C47" s="15" t="inlineStr"/>
-      <c r="D47" s="16" t="inlineStr"/>
+      <c r="C61" s="15" t="inlineStr"/>
+      <c r="D61" s="16" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D47"/>
+  <autoFilter ref="A2:D61"/>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
@@ -3458,7 +3702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V98"/>
+  <dimension ref="A1:V99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3488,7 +3732,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>All 95 publications in the research library. Start with rows marked "Flagship". "In brief" is prefilled where we already had text: correct it if needed. Archive items are hidden by default on the site.</t>
+          <t>All 96 publications in the research library. Start with rows marked "Flagship". "In brief" is prefilled where we already had text: correct it if needed. Archive items are hidden by default on the site.</t>
         </is>
       </c>
     </row>
@@ -8894,12 +9138,12 @@
       </c>
       <c r="B81" s="15" t="inlineStr">
         <is>
-          <t>Contribution (JRC111430)</t>
+          <t>Being a boda isn’t easy</t>
         </is>
       </c>
       <c r="C81" s="15" t="inlineStr">
         <is>
-          <t>European Commission Joint Research Centre</t>
+          <t>Delft University of Technology, MSc thesis</t>
         </is>
       </c>
       <c r="D81" s="15" t="inlineStr">
@@ -8909,32 +9153,36 @@
       </c>
       <c r="E81" s="15" t="inlineStr">
         <is>
-          <t>Ndubuisi</t>
+          <t>Kempers</t>
         </is>
       </c>
       <c r="F81" s="15" t="inlineStr">
         <is>
-          <t>Report</t>
+          <t>thesis</t>
         </is>
       </c>
       <c r="G81" s="15" t="inlineStr">
         <is>
-          <t>01 Green industrialisation &amp; policy</t>
+          <t>04 Innovation, firms &amp; work</t>
         </is>
       </c>
       <c r="H81" s="15" t="inlineStr"/>
-      <c r="I81" s="17" t="inlineStr">
-        <is>
-          <t>https://publications.jrc.ec.europa.eu/repository/handle/JRC111430</t>
+      <c r="I81" s="15" t="inlineStr">
+        <is>
+          <t>TBC</t>
         </is>
       </c>
       <c r="J81" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/contribution-jrc111430</t>
+          <t>https://rita-woad.vercel.app/research/publications/being-a-boda-isnt-easy</t>
         </is>
       </c>
       <c r="K81" s="16" t="inlineStr"/>
-      <c r="L81" s="16" t="inlineStr"/>
+      <c r="L81" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M81" s="16" t="inlineStr"/>
       <c r="N81" s="16" t="inlineStr"/>
       <c r="O81" s="16" t="inlineStr"/>
@@ -8943,7 +9191,11 @@
       <c r="R81" s="16" t="inlineStr"/>
       <c r="S81" s="16" t="inlineStr"/>
       <c r="T81" s="16" t="inlineStr"/>
-      <c r="U81" s="16" t="inlineStr"/>
+      <c r="U81" s="16" t="inlineStr">
+        <is>
+          <t>East Africa</t>
+        </is>
+      </c>
       <c r="V81" s="16" t="inlineStr"/>
     </row>
     <row r="82">
@@ -8952,12 +9204,12 @@
       </c>
       <c r="B82" s="15" t="inlineStr">
         <is>
-          <t>Solid mineral development in Nigeria: evidence from Ebonyi, Ekiti and Taraba states</t>
+          <t>Contribution (JRC111430)</t>
         </is>
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>Centre LSD</t>
+          <t>European Commission Joint Research Centre</t>
         </is>
       </c>
       <c r="D82" s="15" t="inlineStr">
@@ -8977,26 +9229,22 @@
       </c>
       <c r="G82" s="15" t="inlineStr">
         <is>
-          <t>02 Transition minerals &amp; value chains</t>
+          <t>01 Green industrialisation &amp; policy</t>
         </is>
       </c>
       <c r="H82" s="15" t="inlineStr"/>
       <c r="I82" s="17" t="inlineStr">
         <is>
-          <t>https://centrelsd.org/news-and-updates/publications/solid-mineral-development-in-nigeria-evidence-from-ebonyi-ekiti-and-taraba-states</t>
+          <t>https://publications.jrc.ec.europa.eu/repository/handle/JRC111430</t>
         </is>
       </c>
       <c r="J82" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/solid-mineral-development-in-nigeria-evidence-from-ebonyi-ekiti-and</t>
+          <t>https://rita-woad.vercel.app/research/publications/contribution-jrc111430</t>
         </is>
       </c>
       <c r="K82" s="16" t="inlineStr"/>
-      <c r="L82" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="L82" s="16" t="inlineStr"/>
       <c r="M82" s="16" t="inlineStr"/>
       <c r="N82" s="16" t="inlineStr"/>
       <c r="O82" s="16" t="inlineStr"/>
@@ -9005,11 +9253,7 @@
       <c r="R82" s="16" t="inlineStr"/>
       <c r="S82" s="16" t="inlineStr"/>
       <c r="T82" s="16" t="inlineStr"/>
-      <c r="U82" s="16" t="inlineStr">
-        <is>
-          <t>West Africa</t>
-        </is>
-      </c>
+      <c r="U82" s="16" t="inlineStr"/>
       <c r="V82" s="16" t="inlineStr"/>
     </row>
     <row r="83">
@@ -9018,45 +9262,43 @@
       </c>
       <c r="B83" s="15" t="inlineStr">
         <is>
-          <t>PGP for portfolio optimization: application to ESG index family</t>
+          <t>Solid mineral development in Nigeria: evidence from Ebonyi, Ekiti and Taraba states</t>
         </is>
       </c>
       <c r="C83" s="15" t="inlineStr">
         <is>
-          <t>Annals of Operations Research 347(1), 405–417</t>
-        </is>
-      </c>
-      <c r="D83" s="15" t="n">
-        <v>2025</v>
+          <t>Centre LSD</t>
+        </is>
+      </c>
+      <c r="D83" s="15" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
       </c>
       <c r="E83" s="15" t="inlineStr">
         <is>
-          <t>Abid, Urom, Peillex, Karmani, Ndubuisi</t>
+          <t>Ndubuisi</t>
         </is>
       </c>
       <c r="F83" s="15" t="inlineStr">
         <is>
-          <t>Journal article</t>
+          <t>Report</t>
         </is>
       </c>
       <c r="G83" s="15" t="inlineStr">
         <is>
-          <t>01 Green industrialisation &amp; policy</t>
-        </is>
-      </c>
-      <c r="H83" s="15" t="inlineStr">
-        <is>
-          <t>Archive</t>
-        </is>
-      </c>
+          <t>02 Transition minerals &amp; value chains</t>
+        </is>
+      </c>
+      <c r="H83" s="15" t="inlineStr"/>
       <c r="I83" s="17" t="inlineStr">
         <is>
-          <t>https://ideas.repec.org/a/spr/annopr/v347y2025i1d10.1007_s10479-023-05460-w.html</t>
+          <t>https://centrelsd.org/news-and-updates/publications/solid-mineral-development-in-nigeria-evidence-from-ebonyi-ekiti-and-taraba-states</t>
         </is>
       </c>
       <c r="J83" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/pgp-for-portfolio-optimization-esg-index-family</t>
+          <t>https://rita-woad.vercel.app/research/publications/solid-mineral-development-in-nigeria-evidence-from-ebonyi-ekiti-and</t>
         </is>
       </c>
       <c r="K83" s="16" t="inlineStr"/>
@@ -9066,11 +9308,7 @@
         </is>
       </c>
       <c r="M83" s="16" t="inlineStr"/>
-      <c r="N83" s="16" t="inlineStr">
-        <is>
-          <t>Conventional portfolio design assumes Gaussian returns, but asymmetric and heavy-tailed returns call for higher-order moments. The paper proposes a mean-variance-skewness-kurtosis model, optimised with parametrised polynomial goal programming (PGP), to build diversified portfolios.</t>
-        </is>
-      </c>
+      <c r="N83" s="16" t="inlineStr"/>
       <c r="O83" s="16" t="inlineStr"/>
       <c r="P83" s="16" t="inlineStr"/>
       <c r="Q83" s="16" t="inlineStr"/>
@@ -9079,7 +9317,7 @@
       <c r="T83" s="16" t="inlineStr"/>
       <c r="U83" s="16" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>West Africa</t>
         </is>
       </c>
       <c r="V83" s="16" t="inlineStr"/>
@@ -9090,20 +9328,20 @@
       </c>
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>Dependence of green energy markets on big data and other fourth industrial revolution technologies</t>
+          <t>PGP for portfolio optimization: application to ESG index family</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Journal of International Financial Markets, Institutions &amp; Money 96, 102061</t>
+          <t>Annals of Operations Research 347(1), 405–417</t>
         </is>
       </c>
       <c r="D84" s="15" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E84" s="15" t="inlineStr">
         <is>
-          <t>Benkraiem, Guesmi, Ndubuisi, Urom, Vigne</t>
+          <t>Abid, Urom, Peillex, Karmani, Ndubuisi</t>
         </is>
       </c>
       <c r="F84" s="15" t="inlineStr">
@@ -9123,12 +9361,12 @@
       </c>
       <c r="I84" s="17" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S1042443124001276</t>
+          <t>https://ideas.repec.org/a/spr/annopr/v347y2025i1d10.1007_s10479-023-05460-w.html</t>
         </is>
       </c>
       <c r="J84" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/dependence-of-green-energy-markets-on-big-data-and-other-4ir</t>
+          <t>https://rita-woad.vercel.app/research/publications/pgp-for-portfolio-optimization-esg-index-family</t>
         </is>
       </c>
       <c r="K84" s="16" t="inlineStr"/>
@@ -9140,7 +9378,7 @@
       <c r="M84" s="16" t="inlineStr"/>
       <c r="N84" s="16" t="inlineStr">
         <is>
-          <t>The paper analyses dependence and connectedness between fourth industrial revolution technology markets (big data and artificial intelligence, blockchain, financial technology) and global and regional green energy markets, and the roles of market and macroeconomic factors in shock propagation.</t>
+          <t>Conventional portfolio design assumes Gaussian returns, but asymmetric and heavy-tailed returns call for higher-order moments. The paper proposes a mean-variance-skewness-kurtosis model, optimised with parametrised polynomial goal programming (PGP), to build diversified portfolios.</t>
         </is>
       </c>
       <c r="O84" s="16" t="inlineStr"/>
@@ -9162,12 +9400,12 @@
       </c>
       <c r="B85" s="15" t="inlineStr">
         <is>
-          <t>Exploring the coherency and predictability between the stocks of artificial intelligence and energy corporations</t>
+          <t>Dependence of green energy markets on big data and other fourth industrial revolution technologies</t>
         </is>
       </c>
       <c r="C85" s="15" t="inlineStr">
         <is>
-          <t>Financial Innovation 10(1), 128</t>
+          <t>Journal of International Financial Markets, Institutions &amp; Money 96, 102061</t>
         </is>
       </c>
       <c r="D85" s="15" t="n">
@@ -9175,7 +9413,7 @@
       </c>
       <c r="E85" s="15" t="inlineStr">
         <is>
-          <t>Urom, Ndubuisi, Mzoughi, Guesmi</t>
+          <t>Benkraiem, Guesmi, Ndubuisi, Urom, Vigne</t>
         </is>
       </c>
       <c r="F85" s="15" t="inlineStr">
@@ -9195,12 +9433,12 @@
       </c>
       <c r="I85" s="17" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1186/s40854-024-00609-3</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1042443124001276</t>
         </is>
       </c>
       <c r="J85" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/coherency-and-predictability-between-stocks-of-ai-and-energy</t>
+          <t>https://rita-woad.vercel.app/research/publications/dependence-of-green-energy-markets-on-big-data-and-other-4ir</t>
         </is>
       </c>
       <c r="K85" s="16" t="inlineStr"/>
@@ -9212,7 +9450,7 @@
       <c r="M85" s="16" t="inlineStr"/>
       <c r="N85" s="16" t="inlineStr">
         <is>
-          <t>The paper studies links between artificial intelligence investments and eight energy-focused sectors. It finds significant dependence and connectedness, especially over intermediate and long-term investment horizons, and a relationship that has grown stronger since the COVID-19 pandemic.</t>
+          <t>The paper analyses dependence and connectedness between fourth industrial revolution technology markets (big data and artificial intelligence, blockchain, financial technology) and global and regional green energy markets, and the roles of market and macroeconomic factors in shock propagation.</t>
         </is>
       </c>
       <c r="O85" s="16" t="inlineStr"/>
@@ -9234,12 +9472,12 @@
       </c>
       <c r="B86" s="15" t="inlineStr">
         <is>
-          <t>Global macroeconomic factors and the connectedness among NFTs and (un)conventional assets</t>
+          <t>Exploring the coherency and predictability between the stocks of artificial intelligence and energy corporations</t>
         </is>
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>Research in International Business and Finance 71, 102429</t>
+          <t>Financial Innovation 10(1), 128</t>
         </is>
       </c>
       <c r="D86" s="15" t="n">
@@ -9247,7 +9485,7 @@
       </c>
       <c r="E86" s="15" t="inlineStr">
         <is>
-          <t>Urom, Ndubuisi, Guesmi</t>
+          <t>Urom, Ndubuisi, Mzoughi, Guesmi</t>
         </is>
       </c>
       <c r="F86" s="15" t="inlineStr">
@@ -9267,12 +9505,12 @@
       </c>
       <c r="I86" s="17" t="inlineStr">
         <is>
-          <t>https://ideas.repec.org/a/eee/riibaf/v71y2024ics0275531924002228.html</t>
+          <t>https://doi.org/10.1186/s40854-024-00609-3</t>
         </is>
       </c>
       <c r="J86" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/global-macroeconomic-factors-and-connectedness-among-nfts-and-un</t>
+          <t>https://rita-woad.vercel.app/research/publications/coherency-and-predictability-between-stocks-of-ai-and-energy</t>
         </is>
       </c>
       <c r="K86" s="16" t="inlineStr"/>
@@ -9284,7 +9522,7 @@
       <c r="M86" s="16" t="inlineStr"/>
       <c r="N86" s="16" t="inlineStr">
         <is>
-          <t>The paper measures how returns and volatility move between NFTs and conventional and unconventional assets under different market conditions, and tests whether global macroeconomic and geopolitical indicators predict that connectedness.</t>
+          <t>The paper studies links between artificial intelligence investments and eight energy-focused sectors. It finds significant dependence and connectedness, especially over intermediate and long-term investment horizons, and a relationship that has grown stronger since the COVID-19 pandemic.</t>
         </is>
       </c>
       <c r="O86" s="16" t="inlineStr"/>
@@ -9306,20 +9544,20 @@
       </c>
       <c r="B87" s="15" t="inlineStr">
         <is>
-          <t>Dependence and risk spillovers among clean cryptocurrencies prices and media environmental attention</t>
+          <t>Global macroeconomic factors and the connectedness among NFTs and (un)conventional assets</t>
         </is>
       </c>
       <c r="C87" s="15" t="inlineStr">
         <is>
-          <t>Research in International Business and Finance 65, 101953</t>
+          <t>Research in International Business and Finance 71, 102429</t>
         </is>
       </c>
       <c r="D87" s="15" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="E87" s="15" t="inlineStr">
         <is>
-          <t>Ndubuisi, Urom</t>
+          <t>Urom, Ndubuisi, Guesmi</t>
         </is>
       </c>
       <c r="F87" s="15" t="inlineStr">
@@ -9339,12 +9577,12 @@
       </c>
       <c r="I87" s="17" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.ribaf.2023.101953</t>
+          <t>https://ideas.repec.org/a/eee/riibaf/v71y2024ics0275531924002228.html</t>
         </is>
       </c>
       <c r="J87" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/clean-cryptocurrencies-and-media-environmental-attention</t>
+          <t>https://rita-woad.vercel.app/research/publications/global-macroeconomic-factors-and-connectedness-among-nfts-and-un</t>
         </is>
       </c>
       <c r="K87" s="16" t="inlineStr"/>
@@ -9356,7 +9594,7 @@
       <c r="M87" s="16" t="inlineStr"/>
       <c r="N87" s="16" t="inlineStr">
         <is>
-          <t>The study examines the link between media attention to cryptocurrencies' environmental impact and the prices of clean cryptocurrencies. It finds strong connectedness, implying that clean cryptocurrency prices are influenced by attention on cryptocurrency sustainability.</t>
+          <t>The paper measures how returns and volatility move between NFTs and conventional and unconventional assets under different market conditions, and tests whether global macroeconomic and geopolitical indicators predict that connectedness.</t>
         </is>
       </c>
       <c r="O87" s="16" t="inlineStr"/>
@@ -9378,12 +9616,12 @@
       </c>
       <c r="B88" s="15" t="inlineStr">
         <is>
-          <t>Geopolitical risks, global market factors and dependence among regional sustainable investments and commodities</t>
+          <t>Dependence and risk spillovers among clean cryptocurrencies prices and media environmental attention</t>
         </is>
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Quarterly Review of Economics and Finance 91, 94–111</t>
+          <t>Research in International Business and Finance 65, 101953</t>
         </is>
       </c>
       <c r="D88" s="15" t="n">
@@ -9391,7 +9629,7 @@
       </c>
       <c r="E88" s="15" t="inlineStr">
         <is>
-          <t>Urom, Ndubuisi</t>
+          <t>Ndubuisi, Urom</t>
         </is>
       </c>
       <c r="F88" s="15" t="inlineStr">
@@ -9411,12 +9649,12 @@
       </c>
       <c r="I88" s="17" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.qref.2023.07.007</t>
+          <t>https://doi.org/10.1016/j.ribaf.2023.101953</t>
         </is>
       </c>
       <c r="J88" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/geopolitical-risks-global-market-factors-and-dependence-among-regional</t>
+          <t>https://rita-woad.vercel.app/research/publications/clean-cryptocurrencies-and-media-environmental-attention</t>
         </is>
       </c>
       <c r="K88" s="16" t="inlineStr"/>
@@ -9428,7 +9666,7 @@
       <c r="M88" s="16" t="inlineStr"/>
       <c r="N88" s="16" t="inlineStr">
         <is>
-          <t>The paper studies how sustainable investment indices for North America, Europe and Asia-Pacific connect with energy, precious metal and industrial metal commodities. It finds asymmetric connectedness, significantly stronger during extreme downside and upside market conditions.</t>
+          <t>The study examines the link between media attention to cryptocurrencies' environmental impact and the prices of clean cryptocurrencies. It finds strong connectedness, implying that clean cryptocurrency prices are influenced by attention on cryptocurrency sustainability.</t>
         </is>
       </c>
       <c r="O88" s="16" t="inlineStr"/>
@@ -9450,12 +9688,12 @@
       </c>
       <c r="B89" s="15" t="inlineStr">
         <is>
-          <t>Global commodity and equity markets spillovers to Africa during the COVID-19 pandemic</t>
+          <t>Geopolitical risks, global market factors and dependence among regional sustainable investments and commodities</t>
         </is>
       </c>
       <c r="C89" s="15" t="inlineStr">
         <is>
-          <t>Emerging Markets Review 55, 100948</t>
+          <t>Quarterly Review of Economics and Finance 91, 94–111</t>
         </is>
       </c>
       <c r="D89" s="15" t="n">
@@ -9463,7 +9701,7 @@
       </c>
       <c r="E89" s="15" t="inlineStr">
         <is>
-          <t>Urom, Ndubuisi, Del Lo, Yuni</t>
+          <t>Urom, Ndubuisi</t>
         </is>
       </c>
       <c r="F89" s="15" t="inlineStr">
@@ -9483,12 +9721,12 @@
       </c>
       <c r="I89" s="17" t="inlineStr">
         <is>
-          <t>https://ideas.repec.org/a/eee/ememar/v55y2023ics1566014122000656.html</t>
+          <t>https://doi.org/10.1016/j.qref.2023.07.007</t>
         </is>
       </c>
       <c r="J89" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/global-commodity-and-equity-spillovers-to-africa-during-covid-19</t>
+          <t>https://rita-woad.vercel.app/research/publications/geopolitical-risks-global-market-factors-and-dependence-among-regional</t>
         </is>
       </c>
       <c r="K89" s="16" t="inlineStr"/>
@@ -9500,7 +9738,7 @@
       <c r="M89" s="16" t="inlineStr"/>
       <c r="N89" s="16" t="inlineStr">
         <is>
-          <t>The study examines connectedness between 12 African equity markets and global commodity and developed equity markets, with a focus on the peak of the COVID-19 pandemic.</t>
+          <t>The paper studies how sustainable investment indices for North America, Europe and Asia-Pacific connect with energy, precious metal and industrial metal commodities. It finds asymmetric connectedness, significantly stronger during extreme downside and upside market conditions.</t>
         </is>
       </c>
       <c r="O89" s="16" t="inlineStr"/>
@@ -9511,7 +9749,7 @@
       <c r="T89" s="16" t="inlineStr"/>
       <c r="U89" s="16" t="inlineStr">
         <is>
-          <t>Africa-wide</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="V89" s="16" t="inlineStr"/>
@@ -9522,20 +9760,20 @@
       </c>
       <c r="B90" s="15" t="inlineStr">
         <is>
-          <t>Directional predictability and time-frequency spillovers among clean energy sectors and oil price uncertainty</t>
+          <t>Global commodity and equity markets spillovers to Africa during the COVID-19 pandemic</t>
         </is>
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>Quarterly Review of Economics and Finance 85, 326–341</t>
+          <t>Emerging Markets Review 55, 100948</t>
         </is>
       </c>
       <c r="D90" s="15" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="E90" s="15" t="inlineStr">
         <is>
-          <t>Urom, Mzoughi, Ndubuisi, Guesmi</t>
+          <t>Urom, Ndubuisi, Del Lo, Yuni</t>
         </is>
       </c>
       <c r="F90" s="15" t="inlineStr">
@@ -9555,12 +9793,12 @@
       </c>
       <c r="I90" s="17" t="inlineStr">
         <is>
-          <t>https://ideas.repec.org/a/eee/quaeco/v85y2022icp326-341.html</t>
+          <t>https://ideas.repec.org/a/eee/ememar/v55y2023ics1566014122000656.html</t>
         </is>
       </c>
       <c r="J90" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/clean-energy-sectors-and-oil-price-uncertainty</t>
+          <t>https://rita-woad.vercel.app/research/publications/global-commodity-and-equity-spillovers-to-africa-during-covid-19</t>
         </is>
       </c>
       <c r="K90" s="16" t="inlineStr"/>
@@ -9572,7 +9810,7 @@
       <c r="M90" s="16" t="inlineStr"/>
       <c r="N90" s="16" t="inlineStr">
         <is>
-          <t>The paper analyses the dependence between clean energy sectors and oil price uncertainty. Sector responses differ in direction and size depending on the sector, market conditions and investment horizon.</t>
+          <t>The study examines connectedness between 12 African equity markets and global commodity and developed equity markets, with a focus on the peak of the COVID-19 pandemic.</t>
         </is>
       </c>
       <c r="O90" s="16" t="inlineStr"/>
@@ -9583,7 +9821,7 @@
       <c r="T90" s="16" t="inlineStr"/>
       <c r="U90" s="16" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Africa-wide</t>
         </is>
       </c>
       <c r="V90" s="16" t="inlineStr"/>
@@ -9594,12 +9832,12 @@
       </c>
       <c r="B91" s="15" t="inlineStr">
         <is>
-          <t>Dynamic dependence and predictability between volume and return of non-fungible tokens (NFTs): the roles of market factors and geopolitical risks</t>
+          <t>Directional predictability and time-frequency spillovers among clean energy sectors and oil price uncertainty</t>
         </is>
       </c>
       <c r="C91" s="15" t="inlineStr">
         <is>
-          <t>Finance Research Letters 50, 103188</t>
+          <t>Quarterly Review of Economics and Finance 85, 326–341</t>
         </is>
       </c>
       <c r="D91" s="15" t="n">
@@ -9607,7 +9845,7 @@
       </c>
       <c r="E91" s="15" t="inlineStr">
         <is>
-          <t>Urom, Ndubuisi, Guesmi</t>
+          <t>Urom, Mzoughi, Ndubuisi, Guesmi</t>
         </is>
       </c>
       <c r="F91" s="15" t="inlineStr">
@@ -9627,12 +9865,12 @@
       </c>
       <c r="I91" s="17" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.frl.2022.103188</t>
+          <t>https://ideas.repec.org/a/eee/quaeco/v85y2022icp326-341.html</t>
         </is>
       </c>
       <c r="J91" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/nft-volume-and-returns</t>
+          <t>https://rita-woad.vercel.app/research/publications/clean-energy-sectors-and-oil-price-uncertainty</t>
         </is>
       </c>
       <c r="K91" s="16" t="inlineStr"/>
@@ -9644,7 +9882,7 @@
       <c r="M91" s="16" t="inlineStr"/>
       <c r="N91" s="16" t="inlineStr">
         <is>
-          <t>The paper studies the volume–return relationship for the overall NFT market and three sub-markets (Cryptokitties, Cryptopunks and Decentraland). It finds significant dependence between NFT return and volume, weakest for Cryptopunks.</t>
+          <t>The paper analyses the dependence between clean energy sectors and oil price uncertainty. Sector responses differ in direction and size depending on the sector, market conditions and investment horizon.</t>
         </is>
       </c>
       <c r="O91" s="16" t="inlineStr"/>
@@ -9666,12 +9904,12 @@
       </c>
       <c r="B92" s="15" t="inlineStr">
         <is>
-          <t>Dynamic dependence between clean investments and economic policy uncertainty</t>
+          <t>Dynamic dependence and predictability between volume and return of non-fungible tokens (NFTs): the roles of market factors and geopolitical risks</t>
         </is>
       </c>
       <c r="C92" s="15" t="inlineStr">
         <is>
-          <t>UNU-MERIT Working Paper 2022-027</t>
+          <t>Finance Research Letters 50, 103188</t>
         </is>
       </c>
       <c r="D92" s="15" t="n">
@@ -9679,12 +9917,12 @@
       </c>
       <c r="E92" s="15" t="inlineStr">
         <is>
-          <t>Urom, Mzoughi, Ndubuisi, Guesmi</t>
+          <t>Urom, Ndubuisi, Guesmi</t>
         </is>
       </c>
       <c r="F92" s="15" t="inlineStr">
         <is>
-          <t>Working paper</t>
+          <t>Journal article</t>
         </is>
       </c>
       <c r="G92" s="15" t="inlineStr">
@@ -9699,12 +9937,12 @@
       </c>
       <c r="I92" s="17" t="inlineStr">
         <is>
-          <t>https://merit.unu.edu/publications/working-papers/abstract/?id=9378</t>
+          <t>https://doi.org/10.1016/j.frl.2022.103188</t>
         </is>
       </c>
       <c r="J92" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/clean-investments-and-economic-policy-uncertainty</t>
+          <t>https://rita-woad.vercel.app/research/publications/nft-volume-and-returns</t>
         </is>
       </c>
       <c r="K92" s="16" t="inlineStr"/>
@@ -9716,7 +9954,7 @@
       <c r="M92" s="16" t="inlineStr"/>
       <c r="N92" s="16" t="inlineStr">
         <is>
-          <t>The paper examines how clean investments across sectors respond to economic policy uncertainty, using the NASDAQ OMX Green Economy sectoral indexes. Dependence and predictability vary across market conditions and horizons, so the diversification benefits of clean energy stocks depend on sector, market conditions and horizon.</t>
+          <t>The paper studies the volume–return relationship for the overall NFT market and three sub-markets (Cryptokitties, Cryptopunks and Decentraland). It finds significant dependence between NFT return and volume, weakest for Cryptopunks.</t>
         </is>
       </c>
       <c r="O92" s="16" t="inlineStr"/>
@@ -9738,12 +9976,12 @@
       </c>
       <c r="B93" s="15" t="inlineStr">
         <is>
-          <t>Economic sentiment and climate transition during the COVID-19 pandemic</t>
+          <t>Dynamic dependence between clean investments and economic policy uncertainty</t>
         </is>
       </c>
       <c r="C93" s="15" t="inlineStr">
         <is>
-          <t>In Goutte, Guesmi and Urom (eds), Financial Market Dynamics after COVID 19, Springer, ch. 8</t>
+          <t>UNU-MERIT Working Paper 2022-027</t>
         </is>
       </c>
       <c r="D93" s="15" t="n">
@@ -9751,12 +9989,12 @@
       </c>
       <c r="E93" s="15" t="inlineStr">
         <is>
-          <t>Ndubuisi, Yuni, Tingum</t>
+          <t>Urom, Mzoughi, Ndubuisi, Guesmi</t>
         </is>
       </c>
       <c r="F93" s="15" t="inlineStr">
         <is>
-          <t>Book chapter</t>
+          <t>Working paper</t>
         </is>
       </c>
       <c r="G93" s="15" t="inlineStr">
@@ -9771,12 +10009,12 @@
       </c>
       <c r="I93" s="17" t="inlineStr">
         <is>
-          <t>https://www.springerprofessional.de/en/economic-sentiment-and-climate-transition-during-the-covid-19-pa/20350390</t>
+          <t>https://merit.unu.edu/publications/working-papers/abstract/?id=9378</t>
         </is>
       </c>
       <c r="J93" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/economic-sentiment-and-climate-transition-during-covid-19</t>
+          <t>https://rita-woad.vercel.app/research/publications/clean-investments-and-economic-policy-uncertainty</t>
         </is>
       </c>
       <c r="K93" s="16" t="inlineStr"/>
@@ -9788,7 +10026,7 @@
       <c r="M93" s="16" t="inlineStr"/>
       <c r="N93" s="16" t="inlineStr">
         <is>
-          <t>The chapter examines how a newspaper-based US economic sentiment index relates to four climate-themed financial indices after COVID-19 began. Dependence varies across time horizons and market conditions.</t>
+          <t>The paper examines how clean investments across sectors respond to economic policy uncertainty, using the NASDAQ OMX Green Economy sectoral indexes. Dependence and predictability vary across market conditions and horizons, so the diversification benefits of clean energy stocks depend on sector, market conditions and horizon.</t>
         </is>
       </c>
       <c r="O93" s="16" t="inlineStr"/>
@@ -9810,12 +10048,12 @@
       </c>
       <c r="B94" s="15" t="inlineStr">
         <is>
-          <t>How do financial and commodity markets volatility react to real economic activity?</t>
+          <t>Economic sentiment and climate transition during the COVID-19 pandemic</t>
         </is>
       </c>
       <c r="C94" s="15" t="inlineStr">
         <is>
-          <t>Finance Research Letters 47(B), 102733</t>
+          <t>In Goutte, Guesmi and Urom (eds), Financial Market Dynamics after COVID 19, Springer, ch. 8</t>
         </is>
       </c>
       <c r="D94" s="15" t="n">
@@ -9823,12 +10061,12 @@
       </c>
       <c r="E94" s="15" t="inlineStr">
         <is>
-          <t>Urom, Ndubuisi, Guesmi</t>
+          <t>Ndubuisi, Yuni, Tingum</t>
         </is>
       </c>
       <c r="F94" s="15" t="inlineStr">
         <is>
-          <t>Journal article</t>
+          <t>Book chapter</t>
         </is>
       </c>
       <c r="G94" s="15" t="inlineStr">
@@ -9843,12 +10081,12 @@
       </c>
       <c r="I94" s="17" t="inlineStr">
         <is>
-          <t>https://ideas.repec.org/a/eee/finlet/v47y2022ipbs1544612322000563.html</t>
+          <t>https://www.springerprofessional.de/en/economic-sentiment-and-climate-transition-during-the-covid-19-pa/20350390</t>
         </is>
       </c>
       <c r="J94" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/financial-and-commodity-market-volatility-and-real-activity</t>
+          <t>https://rita-woad.vercel.app/research/publications/economic-sentiment-and-climate-transition-during-covid-19</t>
         </is>
       </c>
       <c r="K94" s="16" t="inlineStr"/>
@@ -9860,7 +10098,7 @@
       <c r="M94" s="16" t="inlineStr"/>
       <c r="N94" s="16" t="inlineStr">
         <is>
-          <t>The paper tests lead-lag links and integration between real economic activity and financial and commodity market volatility. Real activity shocks co-move with these markets, but the markets led that co-movement during downturns such as the COVID-19 pandemic.</t>
+          <t>The chapter examines how a newspaper-based US economic sentiment index relates to four climate-themed financial indices after COVID-19 began. Dependence varies across time horizons and market conditions.</t>
         </is>
       </c>
       <c r="O94" s="16" t="inlineStr"/>
@@ -9882,12 +10120,12 @@
       </c>
       <c r="B95" s="15" t="inlineStr">
         <is>
-          <t>Quantile co-movement and dependence between energy-focused sectors and artificial intelligence</t>
+          <t>How do financial and commodity markets volatility react to real economic activity?</t>
         </is>
       </c>
       <c r="C95" s="15" t="inlineStr">
         <is>
-          <t>Technological Forecasting and Social Change 183, 121842</t>
+          <t>Finance Research Letters 47(B), 102733</t>
         </is>
       </c>
       <c r="D95" s="15" t="n">
@@ -9895,7 +10133,7 @@
       </c>
       <c r="E95" s="15" t="inlineStr">
         <is>
-          <t>Urom, Ndubuisi, Guesmi, Benkraien</t>
+          <t>Urom, Ndubuisi, Guesmi</t>
         </is>
       </c>
       <c r="F95" s="15" t="inlineStr">
@@ -9915,12 +10153,12 @@
       </c>
       <c r="I95" s="17" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.techfore.2022.121842</t>
+          <t>https://ideas.repec.org/a/eee/finlet/v47y2022ipbs1544612322000563.html</t>
         </is>
       </c>
       <c r="J95" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/energy-focused-sectors-and-artificial-intelligence</t>
+          <t>https://rita-woad.vercel.app/research/publications/financial-and-commodity-market-volatility-and-real-activity</t>
         </is>
       </c>
       <c r="K95" s="16" t="inlineStr"/>
@@ -9932,7 +10170,7 @@
       <c r="M95" s="16" t="inlineStr"/>
       <c r="N95" s="16" t="inlineStr">
         <is>
-          <t>The paper studies links between artificial intelligence and eight energy-focused sectors. The performance of energy-focused corporations, especially in renewable energy, depends strongly on the performance of AI.</t>
+          <t>The paper tests lead-lag links and integration between real economic activity and financial and commodity market volatility. Real activity shocks co-move with these markets, but the markets led that co-movement during downturns such as the COVID-19 pandemic.</t>
         </is>
       </c>
       <c r="O95" s="16" t="inlineStr"/>
@@ -9954,20 +10192,20 @@
       </c>
       <c r="B96" s="15" t="inlineStr">
         <is>
-          <t>Economic activity, and financial and commodity markets’ shocks: an analysis of implied volatility indexes</t>
+          <t>Quantile co-movement and dependence between energy-focused sectors and artificial intelligence</t>
         </is>
       </c>
       <c r="C96" s="15" t="inlineStr">
         <is>
-          <t>International Economics 165, 51–66</t>
+          <t>Technological Forecasting and Social Change 183, 121842</t>
         </is>
       </c>
       <c r="D96" s="15" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="E96" s="15" t="inlineStr">
         <is>
-          <t>Urom, Ndubuisi, Ozor</t>
+          <t>Urom, Ndubuisi, Guesmi, Benkraien</t>
         </is>
       </c>
       <c r="F96" s="15" t="inlineStr">
@@ -9987,12 +10225,12 @@
       </c>
       <c r="I96" s="17" t="inlineStr">
         <is>
-          <t>https://ideas.repec.org/a/eee/inteco/v165y2021icp51-66.html</t>
+          <t>https://doi.org/10.1016/j.techfore.2022.121842</t>
         </is>
       </c>
       <c r="J96" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/implied-volatility-indexes</t>
+          <t>https://rita-woad.vercel.app/research/publications/energy-focused-sectors-and-artificial-intelligence</t>
         </is>
       </c>
       <c r="K96" s="16" t="inlineStr"/>
@@ -10004,7 +10242,7 @@
       <c r="M96" s="16" t="inlineStr"/>
       <c r="N96" s="16" t="inlineStr">
         <is>
-          <t>The paper examines short- and long-run asymmetric interactions and causality between real economic activity and volatility shocks in stock, energy and gold markets. The relationships are asymmetric at both horizons.</t>
+          <t>The paper studies links between artificial intelligence and eight energy-focused sectors. The performance of energy-focused corporations, especially in renewable energy, depends strongly on the performance of AI.</t>
         </is>
       </c>
       <c r="O96" s="16" t="inlineStr"/>
@@ -10026,12 +10264,12 @@
       </c>
       <c r="B97" s="15" t="inlineStr">
         <is>
-          <t>Global, regional, and national mortality among young people aged 10–24 years, 1950–2019: a systematic analysis for the Global Burden of Disease Study 2019</t>
+          <t>Economic activity, and financial and commodity markets’ shocks: an analysis of implied volatility indexes</t>
         </is>
       </c>
       <c r="C97" s="15" t="inlineStr">
         <is>
-          <t>The Lancet 398(10311), 1593–1618</t>
+          <t>International Economics 165, 51–66</t>
         </is>
       </c>
       <c r="D97" s="15" t="n">
@@ -10039,7 +10277,7 @@
       </c>
       <c r="E97" s="15" t="inlineStr">
         <is>
-          <t>GBD 2019 Adolescent Mortality Collaborators</t>
+          <t>Urom, Ndubuisi, Ozor</t>
         </is>
       </c>
       <c r="F97" s="15" t="inlineStr">
@@ -10049,22 +10287,22 @@
       </c>
       <c r="G97" s="15" t="inlineStr">
         <is>
+          <t>01 Green industrialisation &amp; policy</t>
+        </is>
+      </c>
+      <c r="H97" s="15" t="inlineStr">
+        <is>
           <t>Archive</t>
         </is>
       </c>
-      <c r="H97" s="15" t="inlineStr">
-        <is>
-          <t>Archive</t>
-        </is>
-      </c>
       <c r="I97" s="17" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/S0140-6736(21)01546-4</t>
+          <t>https://ideas.repec.org/a/eee/inteco/v165y2021icp51-66.html</t>
         </is>
       </c>
       <c r="J97" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/global-regional-and-national-mortality-among-young-people-aged-10-24</t>
+          <t>https://rita-woad.vercel.app/research/publications/implied-volatility-indexes</t>
         </is>
       </c>
       <c r="K97" s="16" t="inlineStr"/>
@@ -10076,7 +10314,7 @@
       <c r="M97" s="16" t="inlineStr"/>
       <c r="N97" s="16" t="inlineStr">
         <is>
-          <t>Using GBD 2019 estimates, the study examines deaths and mortality rates among 10–24-year-olds in 204 countries and territories from 1950 to 2019. Variation in adolescent mortality between countries and by sex is widening.</t>
+          <t>The paper examines short- and long-run asymmetric interactions and causality between real economic activity and volatility shocks in stock, energy and gold markets. The relationships are asymmetric at both horizons.</t>
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr"/>
@@ -10098,27 +10336,25 @@
       </c>
       <c r="B98" s="15" t="inlineStr">
         <is>
-          <t>The past and the present: the Nigerian Ebola experience and the Covid-19 pandemic</t>
+          <t>Global, regional, and national mortality among young people aged 10–24 years, 1950–2019: a systematic analysis for the Global Burden of Disease Study 2019</t>
         </is>
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>INCLUDE Platform</t>
-        </is>
-      </c>
-      <c r="D98" s="15" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+          <t>The Lancet 398(10311), 1593–1618</t>
+        </is>
+      </c>
+      <c r="D98" s="15" t="n">
+        <v>2021</v>
       </c>
       <c r="E98" s="15" t="inlineStr">
         <is>
-          <t>Konte, Ndubuisi, Okafor</t>
+          <t>GBD 2019 Adolescent Mortality Collaborators</t>
         </is>
       </c>
       <c r="F98" s="15" t="inlineStr">
         <is>
-          <t>Report</t>
+          <t>Journal article</t>
         </is>
       </c>
       <c r="G98" s="15" t="inlineStr">
@@ -10133,12 +10369,12 @@
       </c>
       <c r="I98" s="17" t="inlineStr">
         <is>
-          <t>https://includeplatform.net/publications/the-past-and-the-present-the-nigerian-ebola-experience-and-the-covid-19-pandemic-2/</t>
+          <t>https://doi.org/10.1016/S0140-6736(21)01546-4</t>
         </is>
       </c>
       <c r="J98" s="17" t="inlineStr">
         <is>
-          <t>https://rita-woad.vercel.app/research/publications/the-past-and-the-present-the-nigerian-ebola-experience-and-covid-19</t>
+          <t>https://rita-woad.vercel.app/research/publications/global-regional-and-national-mortality-among-young-people-aged-10-24</t>
         </is>
       </c>
       <c r="K98" s="16" t="inlineStr"/>
@@ -10150,7 +10386,7 @@
       <c r="M98" s="16" t="inlineStr"/>
       <c r="N98" s="16" t="inlineStr">
         <is>
-          <t>The paper compares Nigeria's success against Ebola with its country-wide response to COVID-19, and assesses which factors may have prevented the country from repeating that success.</t>
+          <t>Using GBD 2019 estimates, the study examines deaths and mortality rates among 10–24-year-olds in 204 countries and territories from 1950 to 2019. Variation in adolescent mortality between countries and by sex is widening.</t>
         </is>
       </c>
       <c r="O98" s="16" t="inlineStr"/>
@@ -10161,21 +10397,95 @@
       <c r="T98" s="16" t="inlineStr"/>
       <c r="U98" s="16" t="inlineStr">
         <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="V98" s="16" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="15" t="n">
+        <v>96</v>
+      </c>
+      <c r="B99" s="15" t="inlineStr">
+        <is>
+          <t>The past and the present: the Nigerian Ebola experience and the Covid-19 pandemic</t>
+        </is>
+      </c>
+      <c r="C99" s="15" t="inlineStr">
+        <is>
+          <t>INCLUDE Platform</t>
+        </is>
+      </c>
+      <c r="D99" s="15" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="E99" s="15" t="inlineStr">
+        <is>
+          <t>Konte, Ndubuisi, Okafor</t>
+        </is>
+      </c>
+      <c r="F99" s="15" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="G99" s="15" t="inlineStr">
+        <is>
+          <t>Archive</t>
+        </is>
+      </c>
+      <c r="H99" s="15" t="inlineStr">
+        <is>
+          <t>Archive</t>
+        </is>
+      </c>
+      <c r="I99" s="17" t="inlineStr">
+        <is>
+          <t>https://includeplatform.net/publications/the-past-and-the-present-the-nigerian-ebola-experience-and-the-covid-19-pandemic-2/</t>
+        </is>
+      </c>
+      <c r="J99" s="17" t="inlineStr">
+        <is>
+          <t>https://rita-woad.vercel.app/research/publications/the-past-and-the-present-the-nigerian-ebola-experience-and-covid-19</t>
+        </is>
+      </c>
+      <c r="K99" s="16" t="inlineStr"/>
+      <c r="L99" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M99" s="16" t="inlineStr"/>
+      <c r="N99" s="16" t="inlineStr">
+        <is>
+          <t>The paper compares Nigeria's success against Ebola with its country-wide response to COVID-19, and assesses which factors may have prevented the country from repeating that success.</t>
+        </is>
+      </c>
+      <c r="O99" s="16" t="inlineStr"/>
+      <c r="P99" s="16" t="inlineStr"/>
+      <c r="Q99" s="16" t="inlineStr"/>
+      <c r="R99" s="16" t="inlineStr"/>
+      <c r="S99" s="16" t="inlineStr"/>
+      <c r="T99" s="16" t="inlineStr"/>
+      <c r="U99" s="16" t="inlineStr">
+        <is>
           <t>West Africa</t>
         </is>
       </c>
-      <c r="V98" s="16" t="inlineStr"/>
+      <c r="V99" s="16" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V98"/>
+  <autoFilter ref="A2:V99"/>
   <mergeCells count="1">
     <mergeCell ref="A1:V1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="L4:L98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L4:L99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Not sure"</formula1>
     </dataValidation>
-    <dataValidation sqref="T4:T98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="T4:T99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Not sure"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10332,42 +10642,43 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId150"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId151"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J83" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J84" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J86" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J87" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J88" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J89" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J90" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J91" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J92" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J93" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J94" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J95" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J96" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J97" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J98" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J83" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J84" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J86" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J87" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J88" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J89" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J90" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J91" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J92" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J93" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J94" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J95" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J96" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J97" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J98" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J99" r:id="rId189"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12179,7 +12490,7 @@
       <c r="I4" s="16" t="inlineStr"/>
       <c r="J4" s="16" t="inlineStr">
         <is>
-          <t>Outages cut jobs, investment and exports; restoring power doesn't restore capabilities, so treat electricity as productive infrastructure.</t>
+          <t>Load shedding has ended, but the damage to manufacturing has not. Drawing on two studies in Energy Policy and Energy Economics, the authors show that outages cut jobs, postponed investment and cost export opportunities, and argue that restoring power does not restore lost capabilities.</t>
         </is>
       </c>
       <c r="K4" s="16" t="inlineStr"/>
@@ -12187,7 +12498,7 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Africa’s mineral strength is wasted if countries don’t work together</t>
+          <t>Africa’s mineral strength is wasted if countries don’t work together – new report</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
@@ -12220,7 +12531,7 @@
       <c r="I5" s="16" t="inlineStr"/>
       <c r="J5" s="16" t="inlineStr">
         <is>
-          <t>No single country has every input; regional coordination turns geology into value chains.</t>
+          <t>Transition minerals are found in 48 African countries, but most still export them raw and capture little value. Drawing on a World Bank–commissioned study, the authors argue that only regional cooperation, shared infrastructure and coordinated policy can turn mineral wealth into regional value chains.</t>
         </is>
       </c>
       <c r="K5" s="16" t="inlineStr"/>
@@ -12257,11 +12568,15 @@
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr"/>
-      <c r="H6" s="16" t="inlineStr"/>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>Please confirm</t>
+        </is>
+      </c>
       <c r="I6" s="16" t="inlineStr"/>
       <c r="J6" s="16" t="inlineStr">
         <is>
-          <t>GVCs create and destroy jobs; gains go to new, small, young firms.</t>
+          <t>Global value chains both create and destroy jobs in South Africa. Net gains come from new, small and young firms entering GVCs, while long-standing participants shed jobs.</t>
         </is>
       </c>
       <c r="K6" s="16" t="inlineStr"/>
@@ -12302,7 +12617,7 @@
       <c r="I7" s="16" t="inlineStr"/>
       <c r="J7" s="16" t="inlineStr">
         <is>
-          <t>Aligned strategies aren't enough; build system coherence around productive bottlenecks.</t>
+          <t>South Africa has one of Africa’s most sophisticated industrial policy architectures, yet transformation remains elusive. Aligned strategies and institutions are not enough: coherence must be built around the productive bottlenecks that hold firms back.</t>
         </is>
       </c>
       <c r="K7" s="16" t="inlineStr"/>
@@ -12339,11 +12654,15 @@
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr"/>
-      <c r="H8" s="16" t="inlineStr"/>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>Please confirm</t>
+        </is>
+      </c>
       <c r="I8" s="16" t="inlineStr"/>
       <c r="J8" s="16" t="inlineStr">
         <is>
-          <t>What matters is technological fit with local capabilities, not where imports come from.</t>
+          <t>Drawing on their study of 52 African countries (2000–2022), the authors argue that what drives structural change is not whether imported inputs come from the North or the South, but how well they fit local capabilities.</t>
         </is>
       </c>
       <c r="K8" s="16" t="inlineStr"/>
@@ -12384,7 +12703,7 @@
       <c r="I9" s="16" t="inlineStr"/>
       <c r="J9" s="16" t="inlineStr">
         <is>
-          <t>Energy reform must become productive reconstruction.</t>
+          <t>Years of power cuts left productive scars: lost manufacturing capacity, investment, export capability and learning that persist after supply improves. A green transition that ignores them may deliver cleaner electricity while reproducing industrial weakness.</t>
         </is>
       </c>
       <c r="K9" s="16" t="inlineStr"/>
@@ -12392,12 +12711,12 @@
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>More about the melody, less about the volume: financing industrial transformation</t>
+          <t>More melody, less volume: financing industrial transformation across Africa</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>OPEC Fund Quarterly</t>
+          <t>OPEC Fund Quarterly, 2026 Q2</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -12425,7 +12744,7 @@
       <c r="I10" s="16" t="inlineStr"/>
       <c r="J10" s="16" t="inlineStr">
         <is>
-          <t>The structure of finance matters: temporal, currency and structural alignment.</t>
+          <t>The debate on financing Africa’s green industrial shift focuses too much on the size of the funding gap. The authors argue the deeper constraint is the structure, quality and purpose of finance, and how well it is aligned with industrial development.</t>
         </is>
       </c>
       <c r="K10" s="16" t="inlineStr"/>
@@ -12438,7 +12757,7 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Growth Research Platform (STEG)</t>
+          <t>STEG Policy Brief, Growth Research Platform (CEPR)</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
@@ -12466,7 +12785,7 @@
       <c r="I11" s="16" t="inlineStr"/>
       <c r="J11" s="16" t="inlineStr">
         <is>
-          <t>Net job gains overall; continuous participants shed jobs.</t>
+          <t>Using data on the universe of formal manufacturing firms in South Africa, the brief finds that joining global value chains brings a net job gain. The gain is driven by firms entering GVCs, largely younger and smaller ones; firms that stay in GVCs shed jobs overall.</t>
         </is>
       </c>
       <c r="K11" s="16" t="inlineStr"/>
@@ -12503,11 +12822,15 @@
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr"/>
-      <c r="H12" s="16" t="inlineStr"/>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>Please confirm</t>
+        </is>
+      </c>
       <c r="I12" s="16" t="inlineStr"/>
       <c r="J12" s="16" t="inlineStr">
         <is>
-          <t>Enter feasible segments (design, ATP, power electronics) collectively via AfCFTA.</t>
+          <t>Africa cannot power its green and digital future without a place in the semiconductor value chain. The brief argues for entering feasible segments, such as chip design, assembly, testing and packaging, and power electronics, collectively through the AfCFTA.</t>
         </is>
       </c>
       <c r="K12" s="16" t="inlineStr"/>
@@ -12520,7 +12843,7 @@
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>UNIDO Policy Brief</t>
+          <t>UNIDO IID Policy Brief 20</t>
         </is>
       </c>
       <c r="C13" s="15" t="inlineStr">
@@ -12535,18 +12858,26 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>Avenyo</t>
+          <t>Asiama, Avenyo, Habiyaremye, Ncube, Tregenna, Donnelly, Lavopa</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>https://lnkd.in/dn7BiAnG</t>
+          <t>https://www.unido.org/publications/policy-briefs</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr"/>
-      <c r="H13" s="16" t="inlineStr"/>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Please confirm</t>
+        </is>
+      </c>
       <c r="I13" s="16" t="inlineStr"/>
-      <c r="J13" s="16" t="inlineStr"/>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Linked to the Africa launch of UNIDO’s Industrial Development Report 2024, the brief assesses Africa’s progress on the industry-related SDGs and argues that industrial policy aligned with the SDGs can drive innovation, decent jobs and climate mitigation.</t>
+        </is>
+      </c>
       <c r="K13" s="16" t="inlineStr"/>
     </row>
     <row r="14">
@@ -12572,7 +12903,7 @@
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>Ndubuisi, Tang, Owusu</t>
+          <t>Owusu, Tang, Ndubuisi</t>
         </is>
       </c>
       <c r="F14" s="17" t="inlineStr">
@@ -12585,7 +12916,7 @@
       <c r="I14" s="16" t="inlineStr"/>
       <c r="J14" s="16" t="inlineStr">
         <is>
-          <t>Chinese FDI raises emissions in resource-intensive sectors; reshape it, don't discourage it.</t>
+          <t>Chinese greenfield manufacturing investment raised industrial carbon emissions in Africa, especially when it went into labour- and resource-intensive manufacturing; the same effect does not appear for OECD investment. The authors argue for reshaping Chinese FDI, not discouraging it.</t>
         </is>
       </c>
       <c r="K14" s="16" t="inlineStr"/>
@@ -12598,7 +12929,7 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>SARChI Industrial Development Policy Brief</t>
+          <t>SARChI Industrial Development Policy Brief 2024-03</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
@@ -12626,7 +12957,7 @@
       <c r="I15" s="16" t="inlineStr"/>
       <c r="J15" s="16" t="inlineStr">
         <is>
-          <t>Capabilities spill over borders through intra-African trade.</t>
+          <t>Little is known about how technological capability shapes industrialisation in Africa. The brief measures capability along four dimensions (preconditions, infrastructure, technology imports and technological effort) and shows that capabilities spill over borders through intra-African trade.</t>
         </is>
       </c>
       <c r="K15" s="16" t="inlineStr"/>
@@ -12634,12 +12965,12 @@
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Catastrophic effects of COVID-19 health expenditure shocks and poverty in Ghana</t>
+          <t>Catastrophic effects of COVID-19 health expenditure shocks and multidimensional poverty in Ghana: what financing mechanisms mattered?</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>AERC Policy Brief</t>
+          <t>AERC Policy Brief AHCV-PB-007</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
@@ -12654,7 +12985,7 @@
       </c>
       <c r="E16" s="15" t="inlineStr">
         <is>
-          <t>Avenyo</t>
+          <t>Ayanore, Avenyo, Osei</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
@@ -12665,18 +12996,22 @@
       <c r="G16" s="16" t="inlineStr"/>
       <c r="H16" s="16" t="inlineStr"/>
       <c r="I16" s="16" t="inlineStr"/>
-      <c r="J16" s="16" t="inlineStr"/>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>More than half of Ghanaian households in the sample spent over 5% of their total expenditure on COVID-19-related health costs. Multidimensional poverty made these catastrophic payments worse, while insurance, remittances and government assistance softened the shock.</t>
+        </is>
+      </c>
       <c r="K16" s="16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Climate change mitigation for late industrialisers: technology intensity in manufacturing</t>
+          <t>Financing digital industrialisation in South Africa: emerging issues</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>CBDS, Copenhagen Business School</t>
+          <t>CCRED-IDTT Policy Brief 2023/5</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
@@ -12686,34 +13021,38 @@
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>2023-02</t>
+          <t>2023-03</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>Avenyo</t>
+          <t>Nyamwena, Avenyo</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>https://research.cbs.dk/files/89602649/elvis_korku_avenyo_et_al_climate_change_mitigation_for_late_industrialisers_publishersversion.pdf</t>
+          <t>https://www.competition.org.za/s/IDTT-2022-2023-PB5_Finance-and-digitalisation.pdf</t>
         </is>
       </c>
       <c r="G17" s="16" t="inlineStr"/>
       <c r="H17" s="16" t="inlineStr"/>
       <c r="I17" s="16" t="inlineStr"/>
-      <c r="J17" s="16" t="inlineStr"/>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Survey evidence from South African manufacturers shows that finance matters for the adoption of digital technologies. The brief sets out the emerging issues in financing digital industrialisation.</t>
+        </is>
+      </c>
       <c r="K17" s="16" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Financing digital industrialisation in South Africa: emerging issues</t>
+          <t>Localisation and industrialisation nexus: lessons for South Africa</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>CCRED-IDTT Policy Brief 2023/05</t>
+          <t>CCRED-IDTT Policy Brief 2023/1</t>
         </is>
       </c>
       <c r="C18" s="15" t="inlineStr">
@@ -12723,38 +13062,38 @@
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>2023-01</t>
+          <t>2023-03</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
         <is>
-          <t>Avenyo</t>
+          <t>Nyamwena, Avenyo, Bosiu</t>
         </is>
       </c>
       <c r="F18" s="17" t="inlineStr">
         <is>
-          <t>https://www.competition.org.za/s/IDTT-2022-2023-PB5_Finance-and-digitalisation.pdf</t>
+          <t>https://www.competition.org.za/s/IDTT-2022-2023-PB1_Localisation-and-Industrialisation-Nexus.pdf</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr"/>
-      <c r="H18" s="16" t="inlineStr">
-        <is>
-          <t>Please confirm</t>
-        </is>
-      </c>
+      <c r="H18" s="16" t="inlineStr"/>
       <c r="I18" s="16" t="inlineStr"/>
-      <c r="J18" s="16" t="inlineStr"/>
+      <c r="J18" s="16" t="inlineStr">
+        <is>
+          <t>A policy brief on how localisation policy connects to industrialisation, and what South Africa can learn from it.</t>
+        </is>
+      </c>
       <c r="K18" s="16" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Localisation and industrialisation nexus: lessons for South Africa</t>
+          <t>Climate change mitigation for late industrialisers: technology intensity in manufacturing</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>CCRED-IDTT Policy Brief 2023/01</t>
+          <t>SARChI Industrial Development Policy Brief 2023-01 (with CBDS, Copenhagen Business School)</t>
         </is>
       </c>
       <c r="C19" s="15" t="inlineStr">
@@ -12764,27 +13103,27 @@
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>2023-01</t>
+          <t>2023-02</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>Avenyo</t>
+          <t>Avenyo, Tregenna</t>
         </is>
       </c>
       <c r="F19" s="17" t="inlineStr">
         <is>
-          <t>https://www.competition.org.za/s/IDTT-2022-2023-PB1_Localisation-and-Industrialisation-Nexus.pdf</t>
+          <t>https://www.uj.ac.za/wp-content/uploads/2021/10/sarchi-id-pb-2023-01-avenyo-e--tregenna-f--january-2023.pdf</t>
         </is>
       </c>
       <c r="G19" s="16" t="inlineStr"/>
-      <c r="H19" s="16" t="inlineStr">
-        <is>
-          <t>Please confirm</t>
-        </is>
-      </c>
+      <c r="H19" s="16" t="inlineStr"/>
       <c r="I19" s="16" t="inlineStr"/>
-      <c r="J19" s="16" t="inlineStr"/>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Late industrialisers need manufacturing to grow, but heavy industrialisation can raise emissions. Drawing on evidence from 56 developing economies, the brief asks whether greener industrial policy, shifting towards higher-technology manufacturing, lets countries industrialise while limiting emissions.</t>
+        </is>
+      </c>
       <c r="K19" s="16" t="inlineStr"/>
     </row>
     <row r="20">
@@ -12805,38 +13144,38 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>2022-01</t>
+          <t>2022-09</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>Avenyo</t>
-        </is>
-      </c>
-      <c r="F20" s="15" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Chisoro-Dube, Avenyo</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>https://www.competition.org.za/s/IDTT5-PB9-Digital-Industrilisation-of-freshness_Final_06072022.pdf</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr"/>
-      <c r="H20" s="16" t="inlineStr">
-        <is>
-          <t>Please confirm</t>
-        </is>
-      </c>
+      <c r="H20" s="16" t="inlineStr"/>
       <c r="I20" s="16" t="inlineStr"/>
-      <c r="J20" s="16" t="inlineStr"/>
+      <c r="J20" s="16" t="inlineStr">
+        <is>
+          <t>A policy brief on how digital technologies are changing fresh-produce value chains in South Africa, part of the Industrial Development Think Tank’s series on climate change and green industrialisation.</t>
+        </is>
+      </c>
       <c r="K20" s="16" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>Digital technology adoption and performance in South African manufacturing: early evidence</t>
+          <t>Implications of COVID-19 on digital transformation in South Africa</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>AERC Policy Brief 2022/004</t>
+          <t>CCRED-IDTT Policy Brief 2022/08</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
@@ -12846,38 +13185,38 @@
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>2022-01</t>
+          <t>2022-07</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>Avenyo</t>
+          <t>Avenyo, Bell, Nyamwena</t>
         </is>
       </c>
       <c r="F21" s="17" t="inlineStr">
         <is>
-          <t>http://publication.aercafricalibrary.org/handle/123456789/3404</t>
+          <t>https://www.competition.org.za/s/IDTT5-PB8-Implications-of-COVID-19-on-digital-transformation-in-South-Africa.pdf</t>
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr"/>
-      <c r="H21" s="16" t="inlineStr">
-        <is>
-          <t>Please confirm</t>
-        </is>
-      </c>
+      <c r="H21" s="16" t="inlineStr"/>
       <c r="I21" s="16" t="inlineStr"/>
-      <c r="J21" s="16" t="inlineStr"/>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Drawing on a survey of 516 South African manufacturing firms, the brief shows how COVID-19 interacted with the shift to digital technologies. Uneven digital uptake weakens the resilience of the firms and industries most exposed to shocks.</t>
+        </is>
+      </c>
       <c r="K21" s="16" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>Implications of COVID-19 on digital transformation in South Africa</t>
+          <t>Digital technology adoption and performance in South African manufacturing firms: early evidence for policy</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>CCRED-IDTT Policy Brief 2022/07</t>
+          <t>AERC Policy Brief</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
@@ -12887,27 +13226,27 @@
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>2022-01</t>
+          <t>2022-03</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>Avenyo</t>
-        </is>
-      </c>
-      <c r="F22" s="15" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Avenyo, Bell</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>https://publication.aercafricalibrary.org/handle/123456789/3404</t>
         </is>
       </c>
       <c r="G22" s="16" t="inlineStr"/>
-      <c r="H22" s="16" t="inlineStr">
-        <is>
-          <t>Please confirm</t>
-        </is>
-      </c>
+      <c r="H22" s="16" t="inlineStr"/>
       <c r="I22" s="16" t="inlineStr"/>
-      <c r="J22" s="16" t="inlineStr"/>
+      <c r="J22" s="16" t="inlineStr">
+        <is>
+          <t>South Africa is a technological follower, and the recovery of its manufacturing may depend on faster digital adoption. The brief shows that the effects of new technologies differ across firms and industries, so digital industrial policy must weigh firm-level factors.</t>
+        </is>
+      </c>
       <c r="K22" s="16" t="inlineStr"/>
     </row>
     <row r="23">
@@ -12944,13 +13283,17 @@
       <c r="G23" s="16" t="inlineStr"/>
       <c r="H23" s="16" t="inlineStr"/>
       <c r="I23" s="16" t="inlineStr"/>
-      <c r="J23" s="16" t="inlineStr"/>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>A survey of 516 South African firms shows the uptake of digital technologies has been slow and uneven. Premature deindustrialisation has left a small, undiversified production base, which makes it harder to meet the basics: connectivity, energy and digital skills.</t>
+        </is>
+      </c>
       <c r="K23" s="16" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>Informal workers in Senegal, Mali and Burkina Faso hit harder by COVID-19</t>
+          <t>Informal workers in Senegal, Mali and Burkina Faso have been hit harder by COVID-19</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
@@ -12970,7 +13313,7 @@
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>Avenyo</t>
+          <t>Balde, Boly, Avenyo</t>
         </is>
       </c>
       <c r="F24" s="17" t="inlineStr">
@@ -12981,7 +13324,11 @@
       <c r="G24" s="16" t="inlineStr"/>
       <c r="H24" s="16" t="inlineStr"/>
       <c r="I24" s="16" t="inlineStr"/>
-      <c r="J24" s="16" t="inlineStr"/>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>A survey of 900 people in Senegal, Mali and Burkina Faso in spring 2020 found that informal workers were more likely to lose their jobs, see their earnings fall and struggle to meet basic needs. The authors set out what this means for social protection and support for small businesses.</t>
+        </is>
+      </c>
       <c r="K24" s="16" t="inlineStr"/>
     </row>
     <row r="25">
@@ -13007,18 +13354,22 @@
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>Avenyo</t>
-        </is>
-      </c>
-      <c r="F25" s="15" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Avenyo, Bell, Nyamwena, Robb</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>https://www.competition.org.za/s/IDTT4_PB_Awakening_industrial_economic_recovery_in_South_Africa_202107.pdf</t>
         </is>
       </c>
       <c r="G25" s="16" t="inlineStr"/>
       <c r="H25" s="16" t="inlineStr"/>
       <c r="I25" s="16" t="inlineStr"/>
-      <c r="J25" s="16" t="inlineStr"/>
+      <c r="J25" s="16" t="inlineStr">
+        <is>
+          <t>A policy brief from the Industrial Development Think Tank on reviving South Africa’s industrial economy after the COVID-19 shock.</t>
+        </is>
+      </c>
       <c r="K25" s="16" t="inlineStr"/>
     </row>
     <row r="26">
@@ -13053,9 +13404,17 @@
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr"/>
-      <c r="H26" s="16" t="inlineStr"/>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>Please confirm</t>
+        </is>
+      </c>
       <c r="I26" s="16" t="inlineStr"/>
-      <c r="J26" s="16" t="inlineStr"/>
+      <c r="J26" s="16" t="inlineStr">
+        <is>
+          <t>For a middle-income technological follower like South Africa, the challenge is to modernise existing capabilities and infrastructure. The Industrial Development Think Tank argues that building digital skills in manufacturing is central to that.</t>
+        </is>
+      </c>
       <c r="K26" s="16" t="inlineStr"/>
     </row>
   </sheetData>
@@ -13085,10 +13444,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13267,7 +13629,7 @@
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>Regionalizing green transition minerals for structural transformation in Africa | Africa’s mineral strength is wasted if countries don’t work together</t>
+          <t>Regionalizing green transition minerals for structural transformation in Africa | Africa’s mineral strength is wasted if countries don’t work together – new report</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr"/>
@@ -13677,7 +14039,11 @@
       </c>
       <c r="H5" s="16" t="inlineStr"/>
       <c r="I5" s="16" t="inlineStr"/>
-      <c r="J5" s="16" t="inlineStr"/>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>African Economic Research Consortium (AERC)</t>
+        </is>
+      </c>
       <c r="K5" s="16" t="inlineStr"/>
       <c r="L5" s="16" t="inlineStr"/>
       <c r="M5" s="16" t="inlineStr"/>
@@ -13723,7 +14089,7 @@
       <c r="I6" s="16" t="inlineStr"/>
       <c r="J6" s="16" t="inlineStr">
         <is>
-          <t>Wits School of Geosciences, Wits Mining Institute, SCIS, SARChI Industrial Development</t>
+          <t>Southern Centre for Inequality Studies (SCIS), Wits, Wits School of Geosciences, Wits Mining Institute, SARChI Industrial Development, University of Johannesburg</t>
         </is>
       </c>
       <c r="K6" s="16" t="inlineStr"/>
@@ -13749,7 +14115,7 @@
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -13768,8 +14134,14 @@
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr"/>
-      <c r="I7" s="16" t="inlineStr"/>
-      <c r="J7" s="16" t="inlineStr"/>
+      <c r="I7" s="16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>African Economic Research Consortium (AERC)</t>
+        </is>
+      </c>
       <c r="K7" s="16" t="inlineStr"/>
       <c r="L7" s="16" t="inlineStr"/>
       <c r="M7" s="16" t="inlineStr"/>
@@ -13793,7 +14165,7 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -13812,8 +14184,14 @@
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr"/>
-      <c r="I8" s="16" t="inlineStr"/>
-      <c r="J8" s="16" t="inlineStr"/>
+      <c r="I8" s="16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>UNU-WIDER, SA-TIED</t>
+        </is>
+      </c>
       <c r="K8" s="16" t="inlineStr"/>
       <c r="L8" s="16" t="inlineStr"/>
       <c r="M8" s="16" t="inlineStr"/>
@@ -13837,7 +14215,7 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
@@ -13856,8 +14234,14 @@
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr"/>
-      <c r="I9" s="16" t="inlineStr"/>
-      <c r="J9" s="16" t="inlineStr"/>
+      <c r="I9" s="16" t="n">
+        <v>2020</v>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>UNU-WIDER, SA-TIED, National Treasury, South African Revenue Service</t>
+        </is>
+      </c>
       <c r="K9" s="16" t="inlineStr"/>
       <c r="L9" s="16" t="inlineStr"/>
       <c r="M9" s="16" t="inlineStr"/>
@@ -13881,7 +14265,7 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -13900,8 +14284,14 @@
         </is>
       </c>
       <c r="H10" s="16" t="inlineStr"/>
-      <c r="I10" s="16" t="inlineStr"/>
-      <c r="J10" s="16" t="inlineStr"/>
+      <c r="I10" s="16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="J10" s="16" t="inlineStr">
+        <is>
+          <t>African Economic Research Consortium (AERC)</t>
+        </is>
+      </c>
       <c r="K10" s="16" t="inlineStr"/>
       <c r="L10" s="16" t="inlineStr"/>
       <c r="M10" s="16" t="inlineStr"/>
@@ -13947,7 +14337,11 @@
       <c r="I11" s="16" t="n">
         <v>2025</v>
       </c>
-      <c r="J11" s="16" t="inlineStr"/>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>UNIDO</t>
+        </is>
+      </c>
       <c r="K11" s="16" t="inlineStr"/>
       <c r="L11" s="16" t="inlineStr"/>
       <c r="M11" s="16" t="inlineStr"/>
@@ -13993,7 +14387,11 @@
       <c r="I12" s="16" t="n">
         <v>2025</v>
       </c>
-      <c r="J12" s="16" t="inlineStr"/>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>World Bank, Office of the Chief Economist for the Africa Region</t>
+        </is>
+      </c>
       <c r="K12" s="16" t="inlineStr"/>
       <c r="L12" s="16" t="inlineStr"/>
       <c r="M12" s="16" t="inlineStr"/>
@@ -14017,7 +14415,7 @@
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>2020–2025</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -14035,9 +14433,17 @@
           <t>https://rita-woad.vercel.app/research/projects/research-network-sustainable-supply-chains</t>
         </is>
       </c>
-      <c r="H13" s="16" t="inlineStr"/>
-      <c r="I13" s="16" t="inlineStr"/>
-      <c r="J13" s="16" t="inlineStr"/>
+      <c r="H13" s="16" t="n">
+        <v>2020</v>
+      </c>
+      <c r="I13" s="16" t="n">
+        <v>2025</v>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>German Development Institute (DIE/IDOS), German Institute for International and Security Affairs (SWP), GIGA, Kiel Institute for the World Economy (IfW)</t>
+        </is>
+      </c>
       <c r="K13" s="16" t="inlineStr"/>
       <c r="L13" s="16" t="inlineStr"/>
       <c r="M13" s="16" t="inlineStr"/>
@@ -14083,7 +14489,11 @@
       <c r="I14" s="16" t="n">
         <v>2023</v>
       </c>
-      <c r="J14" s="16" t="inlineStr"/>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>UNCTAD</t>
+        </is>
+      </c>
       <c r="K14" s="16" t="inlineStr"/>
       <c r="L14" s="16" t="inlineStr"/>
       <c r="M14" s="16" t="inlineStr"/>
@@ -14127,13 +14537,13 @@
       </c>
       <c r="H15" s="16" t="inlineStr"/>
       <c r="I15" s="16" t="inlineStr"/>
-      <c r="J15" s="16" t="inlineStr"/>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Department of Science and Innovation, South Africa</t>
+        </is>
+      </c>
       <c r="K15" s="16" t="inlineStr"/>
-      <c r="L15" s="16" t="inlineStr">
-        <is>
-          <t>Co-PI</t>
-        </is>
-      </c>
+      <c r="L15" s="16" t="inlineStr"/>
       <c r="M15" s="16" t="inlineStr"/>
       <c r="N15" s="16" t="inlineStr"/>
     </row>
@@ -14155,7 +14565,7 @@
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
@@ -14173,9 +14583,17 @@
           <t>https://rita-woad.vercel.app/research/projects/services-sector-acceleration</t>
         </is>
       </c>
-      <c r="H16" s="16" t="inlineStr"/>
-      <c r="I16" s="16" t="inlineStr"/>
-      <c r="J16" s="16" t="inlineStr"/>
+      <c r="H16" s="16" t="n">
+        <v>2023</v>
+      </c>
+      <c r="I16" s="16" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>UNU-WIDER, Groningen Growth and Development Centre (GGDC)</t>
+        </is>
+      </c>
       <c r="K16" s="16" t="inlineStr"/>
       <c r="L16" s="16" t="inlineStr"/>
       <c r="M16" s="16" t="inlineStr"/>
@@ -14199,7 +14617,7 @@
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
@@ -14218,8 +14636,14 @@
         </is>
       </c>
       <c r="H17" s="16" t="inlineStr"/>
-      <c r="I17" s="16" t="inlineStr"/>
-      <c r="J17" s="16" t="inlineStr"/>
+      <c r="I17" s="16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Africa Policy Research Institute (APRI)</t>
+        </is>
+      </c>
       <c r="K17" s="16" t="inlineStr"/>
       <c r="L17" s="16" t="inlineStr"/>
       <c r="M17" s="16" t="inlineStr"/>
@@ -14243,7 +14667,7 @@
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
@@ -14262,8 +14686,14 @@
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr"/>
-      <c r="I18" s="16" t="inlineStr"/>
-      <c r="J18" s="16" t="inlineStr"/>
+      <c r="I18" s="16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J18" s="16" t="inlineStr">
+        <is>
+          <t>African Center for Economic Transformation (ACET)</t>
+        </is>
+      </c>
       <c r="K18" s="16" t="inlineStr"/>
       <c r="L18" s="16" t="inlineStr"/>
       <c r="M18" s="16" t="inlineStr"/>

</xml_diff>